<commit_message>
feat: add project material database sheet
</commit_message>
<xml_diff>
--- a/translators/translator_at_v2.0.0.xlsx
+++ b/translators/translator_at_v2.0.0.xlsx
@@ -558,15 +558,13 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Version 2.0.0 | October 2026 | pre-release</t>
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="22" t="inlineStr">
         <is>
@@ -616,47 +614,43 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Authors: Nicole Di Santo¹, Martin Röck²</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Contributors: Karen Scrivener¹, Vanderley John³, Zuhaib Batra¹</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>1. GBDI Global Building Data Initiative, EPFL LMC, Lausanne, Switzerland</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>2. RISE Institute for Regenerative Spatial Systems Science, Vienna, Austria</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>3. University of São Paulo, São Paulo, Brazil</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Contacts:</t>
         </is>
@@ -676,16 +670,15 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Parser and code implementation with support of ENAC-IT4R, EPFL, Lausanne.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>GitHub repository:</t>
         </is>
@@ -2851,7 +2844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="11" min="1" max="4"/>
@@ -2972,41 +2965,67 @@
     <row r="4" ht="15" customHeight="1" s="12">
       <c r="A4" s="11" t="inlineStr">
         <is>
+          <t>Project Material Database</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Project Material Database</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>horizontal</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="12">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
           <t>Summen</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>LCA Result (Wide)</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>horizontal</t>
         </is>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H5" s="11" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="12">
-      <c r="B5" s="11" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>LCA Result (Tall)</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>horizontal</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D6" s="11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fill automatic fields
</commit_message>
<xml_diff>
--- a/translators/translator_at_v2.0.0.xlsx
+++ b/translators/translator_at_v2.0.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="30"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" state="visible" r:id="rId3"/>
@@ -38,6 +38,7 @@
     <sheet name="BiogenicCarbonAccounting" sheetId="28" state="visible" r:id="rId30"/>
     <sheet name="MaterialQuantitiesSource" sheetId="29" state="visible" r:id="rId31"/>
     <sheet name="AboveBelowGround" sheetId="30" state="visible" r:id="rId32"/>
+    <sheet name="FloorLevel" sheetId="31" state="visible" r:id="rId33"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3635" uniqueCount="2391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3647" uniqueCount="2400">
   <si>
     <t xml:space="preserve">OpenBDF - Open Building Data Format</t>
   </si>
@@ -7885,6 +7886,33 @@
   </si>
   <si>
     <t xml:space="preserve">@REGEX^Untergeschoß</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenBDF floor level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@INT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erdgeschoss, ground floor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ground floor, Austrian spelling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@REGEX^KG.*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kellergeschoss, basement storey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Untergeschoss, basement storey</t>
   </si>
 </sst>
 </file>
@@ -15710,6 +15738,89 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="80"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>2391</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2392</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>2393</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>2394</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>2395</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>2380</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>2396</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>2397</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>2398</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>2389</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>2399</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>